<commit_message>
Obtengo predicciones para los proximos 15 dias
</commit_message>
<xml_diff>
--- a/data/england/p6_deployment/data_preparation/clean_data/df_match_player_cleaned.xlsx
+++ b/data/england/p6_deployment/data_preparation/clean_data/df_match_player_cleaned.xlsx
@@ -425,391 +425,321 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:A56"/>
+  <dimension ref="A2:A46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Kl1AOZN9</t>
+          <t>8j9FTL56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>t4kJMDhM</t>
+          <t>U5cORazJ</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>CntkHiGq</t>
+          <t>dCkAk3SP</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>hdlcFVpd</t>
+          <t>lAUlrLKa</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>pjyqwZx3</t>
+          <t>fNaktakC</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>tIUiyD7F</t>
+          <t>2m3cvwKO</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>nHdPI4il</t>
+          <t>2g67Vsyf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>8WpYGrM0</t>
+          <t>6RCbX36s</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>fmqtFMjD</t>
+          <t>61T7bt5t</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>AeRSxQrK</t>
+          <t>GdWtpsjm</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>8j9FTL56</t>
+          <t>ERWFdKZh</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>U5cORazJ</t>
+          <t>8QPOfb45</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>dCkAk3SP</t>
+          <t>x6HuiG3U</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>lAUlrLKa</t>
+          <t>SUdkBJln</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>fNaktakC</t>
+          <t>lpob9cJb</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>2m3cvwKO</t>
+          <t>2Fanm72d</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>2g67Vsyf</t>
+          <t>INsZAAf3</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>6RCbX36s</t>
+          <t>tvOWhxZH</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>61T7bt5t</t>
+          <t>U11vkTXq</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>GdWtpsjm</t>
+          <t>z1q67ylB</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>OMDVg8x9</t>
+          <t>rRQ6H30k</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>jXcAnQUr</t>
+          <t>dUjtW2Fr</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>fRe0c20b</t>
+          <t>MFnpCm7C</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>CnnJp4ae</t>
+          <t>UsklUtpe</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>bw1zAKS6</t>
+          <t>ddFjPf2b</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>GINCsvmn</t>
+          <t>Sh9BS8ig</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>x6klsVh3</t>
+          <t>dAfPwfHi</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>b3pRrrU7</t>
+          <t>pWQ6LC1N</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>WfkfPdXH</t>
+          <t>jiUEFsV1</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>SMr3Nz2U</t>
+          <t>dY0SOQjI</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>xYBLuIHb</t>
+          <t>hO8aNYWA</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>6os5wmhS</t>
+          <t>vDA9yPiL</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>Kl7vhn7L</t>
+          <t>hzeTFV7m</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>nw6fJO5K</t>
+          <t>Q9rcSKE7</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>bHPacsq1</t>
+          <t>zJCJQnM5</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>MwmHgKaN</t>
+          <t>QkntzCGG</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>lQl9etVA</t>
+          <t>Wn71woN8</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>KWD8eLDD</t>
+          <t>EkqxE9x0</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>xUXzYQFk</t>
+          <t>GEugARyP</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>CCV9JR0d</t>
+          <t>U32wGjPp</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>bsinRI25</t>
+          <t>hGzqjO6E</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>GbaVU03t</t>
+          <t>OrHrRGXo</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>tOTmlbNp</t>
+          <t>WQF2UUMt</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>nPQL4PjR</t>
+          <t>rkazN4LU</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>pWhdu9NF</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="1" t="inlineStr">
-        <is>
-          <t>6NnRD2Ts</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="1" t="inlineStr">
-        <is>
-          <t>2FcwTvYh</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="1" t="inlineStr">
-        <is>
-          <t>EBSD6oME</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="1" t="inlineStr">
-        <is>
-          <t>WSQqW4p2</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="1" t="inlineStr">
-        <is>
-          <t>vaX1LmWq</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="1" t="inlineStr">
-        <is>
-          <t>n1hhaOVo</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="1" t="inlineStr">
-        <is>
-          <t>vyoZBtbf</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="1" t="inlineStr">
-        <is>
-          <t>634r8bcJ</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="1" t="inlineStr">
-        <is>
-          <t>pbFTwdnB</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="1" t="inlineStr">
-        <is>
-          <t>697ha3El</t>
+          <t>hxlYyYo4</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Recolección de partidos de los próximos 15 días con nuevos modelos en ITA y GER.
</commit_message>
<xml_diff>
--- a/data/england/p6_deployment/data_preparation/clean_data/df_match_player_cleaned.xlsx
+++ b/data/england/p6_deployment/data_preparation/clean_data/df_match_player_cleaned.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:A46"/>
+  <dimension ref="A2:A21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -568,181 +568,6 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>rRQ6H30k</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="1" t="inlineStr">
-        <is>
-          <t>dUjtW2Fr</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>MFnpCm7C</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="1" t="inlineStr">
-        <is>
-          <t>UsklUtpe</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="1" t="inlineStr">
-        <is>
-          <t>ddFjPf2b</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="1" t="inlineStr">
-        <is>
-          <t>Sh9BS8ig</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="1" t="inlineStr">
-        <is>
-          <t>dAfPwfHi</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="1" t="inlineStr">
-        <is>
-          <t>pWQ6LC1N</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="1" t="inlineStr">
-        <is>
-          <t>jiUEFsV1</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="1" t="inlineStr">
-        <is>
-          <t>dY0SOQjI</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="1" t="inlineStr">
-        <is>
-          <t>hO8aNYWA</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="1" t="inlineStr">
-        <is>
-          <t>vDA9yPiL</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="1" t="inlineStr">
-        <is>
-          <t>hzeTFV7m</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="1" t="inlineStr">
-        <is>
-          <t>Q9rcSKE7</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="1" t="inlineStr">
-        <is>
-          <t>zJCJQnM5</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="1" t="inlineStr">
-        <is>
-          <t>QkntzCGG</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="1" t="inlineStr">
-        <is>
-          <t>Wn71woN8</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="1" t="inlineStr">
-        <is>
-          <t>EkqxE9x0</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="1" t="inlineStr">
-        <is>
-          <t>GEugARyP</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="1" t="inlineStr">
-        <is>
-          <t>U32wGjPp</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="1" t="inlineStr">
-        <is>
-          <t>hGzqjO6E</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="1" t="inlineStr">
-        <is>
-          <t>OrHrRGXo</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="1" t="inlineStr">
-        <is>
-          <t>WQF2UUMt</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="1" t="inlineStr">
-        <is>
-          <t>rkazN4LU</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="1" t="inlineStr">
-        <is>
-          <t>hxlYyYo4</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizo predicciones.xlsx para n_days=3
</commit_message>
<xml_diff>
--- a/data/england/p6_deployment/data_preparation/clean_data/df_match_player_cleaned.xlsx
+++ b/data/england/p6_deployment/data_preparation/clean_data/df_match_player_cleaned.xlsx
@@ -425,146 +425,238 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:A21"/>
+  <dimension ref="A1:Q3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>id_player_miss_home_1</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>player_name_miss_home_1</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>id_player_miss_away_1</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>player_name_miss_away_1</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>id_player_miss_away_2</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>player_name_miss_away_2</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>id_player_miss_away_3</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>player_name_miss_away_3</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>id_player_miss_away_4</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>player_name_miss_away_4</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>id_player_miss_away_5</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>player_name_miss_away_5</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>id_player_miss_home_2</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>player_name_miss_home_2</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>id_player_miss_home_3</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>player_name_miss_home_3</t>
+        </is>
+      </c>
+    </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>2kGeEq1e</t>
-        </is>
-      </c>
+          <t>AFJ3CNV7</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>K82Dz773</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>richarlison</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>QFt86bm1</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>merino mikel</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>ID32TGhp</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>odegaard martin</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>zkQ8Cm6n</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>rice declan</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Qm0l3aod</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>tierney kieran</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>OSNvjZSP</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>tomiyasu takehiro</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>2TvL16Hk</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>beYTapn2</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>jkLFNmv9</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>AiyHLR8L</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>tzSnG5Wr</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>Wplk7SgS</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>AVat9lPF</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>AFJ3CNV7</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
           <t>Of1jzRNE</t>
         </is>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>C0axT3Xo</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>d8abY4hR</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>pYXoP0FD</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>xtzXn47K</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>dQG3srVs</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>Q58Kw0U6</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>W2BSyvaJ</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>OIqwRMp1</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>GhtVSrGl</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>UwFBuMaf</t>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>dU6MwnBl</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>chiwome leon</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>nRvavHmI</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>botman sven</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0fPiq0ST</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>lascelles jamaal</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>nR5TcNGS</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>miley lewis</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>YwKMvtoh</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>wilson callum</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>jDBbY3US</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>david gonzalez</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>8Wq79aVu</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>kalajdzic sasa</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cambio modelo de ITA (XGBoost con mas hiper en GridSearch) y actualizo predicciones.xlsx
</commit_message>
<xml_diff>
--- a/data/england/p6_deployment/data_preparation/clean_data/df_match_player_cleaned.xlsx
+++ b/data/england/p6_deployment/data_preparation/clean_data/df_match_player_cleaned.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y21"/>
+  <dimension ref="A1:W21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -537,16 +537,6 @@
       <c r="W1" s="1" t="inlineStr">
         <is>
           <t>player_name_miss_home_5</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>id_player_miss_home_6</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>player_name_miss_home_6</t>
         </is>
       </c>
     </row>
@@ -602,8 +592,6 @@
       <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr"/>
       <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
-      <c r="Y2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -631,20 +619,36 @@
           <t>cuenca jorge</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>nwu2UvUA</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>lukic sasa</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
+          <t>4CQLQWTa</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>konsa ezri</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
           <t>rgGnzD2e</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>mcginn john</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
@@ -657,8 +661,6 @@
       <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr"/>
       <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
-      <c r="Y3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -668,48 +670,64 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>bkbKtyxR</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>al hamadi ali</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>MwredEF5</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>donacien janoi</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Aw3OUCyR</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>luongo massimo</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>0rnu9an9</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>broja armando</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>SI6IcTms</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>chermiti</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
         <is>
           <t>l21PrfBG</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>tuanzebe axel</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>0rnu9an9</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>broja armando</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>SI6IcTms</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>chermiti</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
@@ -720,8 +738,6 @@
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr"/>
       <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
-      <c r="Y4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -831,8 +847,6 @@
       </c>
       <c r="V5" t="inlineStr"/>
       <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr"/>
-      <c r="Y5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -852,22 +866,22 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>p41IV42c</t>
+          <t>0fPiq0ST</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>isak alexander</t>
+          <t>lascelles jamaal</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0fPiq0ST</t>
+          <t>nR5TcNGS</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>lascelles jamaal</t>
+          <t>miley lewis</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -882,60 +896,50 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
+          <t>0rGKAqEi</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>march solomon</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>GMqWRFGS</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>trippier kieran</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
           <t>AZOU76Ou</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>o riley matthew</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>nR5TcNGS</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>miley lewis</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>WG59HGIH</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>van hecke jan paul</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>IJd0tRWR</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>webster adam</t>
+        </is>
+      </c>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>GMqWRFGS</t>
-        </is>
-      </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>trippier kieran</t>
-        </is>
-      </c>
-      <c r="X6" t="inlineStr">
-        <is>
-          <t>YwKMvtoh</t>
-        </is>
-      </c>
-      <c r="Y6" t="inlineStr">
-        <is>
-          <t>wilson callum</t>
-        </is>
-      </c>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -965,12 +969,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>EksgGjXe</t>
+          <t>lxFOy0k5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>sulemana kamal deen</t>
+          <t>stephens jack</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -993,8 +997,16 @@
           <t>daka patson</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2L76lB8m</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>stewart ross</t>
+        </is>
+      </c>
       <c r="N7" t="inlineStr">
         <is>
           <t>I126P2TJ</t>
@@ -1021,8 +1033,6 @@
       <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr"/>
       <c r="W7" t="inlineStr"/>
-      <c r="X7" t="inlineStr"/>
-      <c r="Y7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -1038,22 +1048,22 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
+          <t>dbGArTGd</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>neto</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
           <t>ID32TGhp</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>odegaard martin</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>08NLEo06</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>saka bukayo</t>
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
@@ -1084,8 +1094,6 @@
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr"/>
       <c r="W8" t="inlineStr"/>
-      <c r="X8" t="inlineStr"/>
-      <c r="Y8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
@@ -1093,30 +1101,100 @@
           <t>SSZaQ4Ct</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>dU6MwnBl</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>chiwome leon</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>jDBbY3US</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>david gonzalez</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>8Wq79aVu</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>kalajdzic sasa</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>6LBvaQoh</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>ake nathan</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>GzxuaXeQ</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>bobb oscar</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>AeyqOcqS</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>mosquera yerson</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>MsPs6OI5</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>de bruyne kevin</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>K0G8DB00</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>rodri</t>
+        </is>
+      </c>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr"/>
-      <c r="V9" t="inlineStr"/>
-      <c r="W9" t="inlineStr"/>
-      <c r="X9" t="inlineStr"/>
-      <c r="Y9" t="inlineStr"/>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>I3feMxCH</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>traore boubacar</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
@@ -1146,8 +1224,6 @@
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr"/>
       <c r="W10" t="inlineStr"/>
-      <c r="X10" t="inlineStr"/>
-      <c r="Y10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
@@ -1177,8 +1253,6 @@
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr"/>
       <c r="W11" t="inlineStr"/>
-      <c r="X11" t="inlineStr"/>
-      <c r="Y11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
@@ -1208,8 +1282,6 @@
       <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr"/>
       <c r="W12" t="inlineStr"/>
-      <c r="X12" t="inlineStr"/>
-      <c r="Y12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
@@ -1239,8 +1311,6 @@
       <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr"/>
       <c r="W13" t="inlineStr"/>
-      <c r="X13" t="inlineStr"/>
-      <c r="Y13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
@@ -1270,8 +1340,6 @@
       <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr"/>
       <c r="W14" t="inlineStr"/>
-      <c r="X14" t="inlineStr"/>
-      <c r="Y14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
@@ -1301,8 +1369,6 @@
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr"/>
       <c r="W15" t="inlineStr"/>
-      <c r="X15" t="inlineStr"/>
-      <c r="Y15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
@@ -1332,8 +1398,6 @@
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr"/>
       <c r="W16" t="inlineStr"/>
-      <c r="X16" t="inlineStr"/>
-      <c r="Y16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
@@ -1363,8 +1427,6 @@
       <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr"/>
       <c r="W17" t="inlineStr"/>
-      <c r="X17" t="inlineStr"/>
-      <c r="Y17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
@@ -1394,8 +1456,6 @@
       <c r="U18" t="inlineStr"/>
       <c r="V18" t="inlineStr"/>
       <c r="W18" t="inlineStr"/>
-      <c r="X18" t="inlineStr"/>
-      <c r="Y18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
@@ -1425,8 +1485,6 @@
       <c r="U19" t="inlineStr"/>
       <c r="V19" t="inlineStr"/>
       <c r="W19" t="inlineStr"/>
-      <c r="X19" t="inlineStr"/>
-      <c r="Y19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
@@ -1456,8 +1514,6 @@
       <c r="U20" t="inlineStr"/>
       <c r="V20" t="inlineStr"/>
       <c r="W20" t="inlineStr"/>
-      <c r="X20" t="inlineStr"/>
-      <c r="Y20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
@@ -1487,8 +1543,6 @@
       <c r="U21" t="inlineStr"/>
       <c r="V21" t="inlineStr"/>
       <c r="W21" t="inlineStr"/>
-      <c r="X21" t="inlineStr"/>
-      <c r="Y21" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>